<commit_message>
Updated POL_grids_syn_5 model - 2025-11-19 13:25
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF144F31-57A1-433F-85B4-63B47B78E067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{479ECF1D-3BA6-4E5D-87C4-74D2FD9F76AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1606,94 +1606,94 @@
     <t>p_sol20</t>
   </si>
   <si>
-    <t>p_won21</t>
-  </si>
-  <si>
-    <t>p_won22</t>
-  </si>
-  <si>
-    <t>p_won23</t>
-  </si>
-  <si>
-    <t>p_won24</t>
-  </si>
-  <si>
-    <t>p_won25</t>
-  </si>
-  <si>
-    <t>p_won26</t>
-  </si>
-  <si>
-    <t>p_won27</t>
-  </si>
-  <si>
-    <t>p_won28</t>
-  </si>
-  <si>
-    <t>p_won29</t>
-  </si>
-  <si>
-    <t>p_won30</t>
-  </si>
-  <si>
-    <t>p_won31</t>
-  </si>
-  <si>
-    <t>p_won32</t>
-  </si>
-  <si>
-    <t>p_won33</t>
-  </si>
-  <si>
-    <t>p_won34</t>
-  </si>
-  <si>
-    <t>p_won35</t>
-  </si>
-  <si>
-    <t>p_won36</t>
-  </si>
-  <si>
-    <t>p_won37</t>
-  </si>
-  <si>
-    <t>p_won38</t>
-  </si>
-  <si>
-    <t>p_won39</t>
-  </si>
-  <si>
-    <t>p_won40</t>
-  </si>
-  <si>
-    <t>p_wof41</t>
-  </si>
-  <si>
-    <t>p_wof42</t>
-  </si>
-  <si>
-    <t>p_wof43</t>
-  </si>
-  <si>
-    <t>p_wof44</t>
-  </si>
-  <si>
-    <t>p_wof45</t>
-  </si>
-  <si>
-    <t>p_wof46</t>
-  </si>
-  <si>
-    <t>p_wof47</t>
-  </si>
-  <si>
-    <t>p_wof48</t>
-  </si>
-  <si>
-    <t>p_wof49</t>
-  </si>
-  <si>
-    <t>p_wof50</t>
+    <t>p_won1</t>
+  </si>
+  <si>
+    <t>p_won2</t>
+  </si>
+  <si>
+    <t>p_won3</t>
+  </si>
+  <si>
+    <t>p_won4</t>
+  </si>
+  <si>
+    <t>p_won5</t>
+  </si>
+  <si>
+    <t>p_won6</t>
+  </si>
+  <si>
+    <t>p_won7</t>
+  </si>
+  <si>
+    <t>p_won8</t>
+  </si>
+  <si>
+    <t>p_won9</t>
+  </si>
+  <si>
+    <t>p_won10</t>
+  </si>
+  <si>
+    <t>p_won11</t>
+  </si>
+  <si>
+    <t>p_won12</t>
+  </si>
+  <si>
+    <t>p_won13</t>
+  </si>
+  <si>
+    <t>p_won14</t>
+  </si>
+  <si>
+    <t>p_won15</t>
+  </si>
+  <si>
+    <t>p_won16</t>
+  </si>
+  <si>
+    <t>p_won17</t>
+  </si>
+  <si>
+    <t>p_won18</t>
+  </si>
+  <si>
+    <t>p_won19</t>
+  </si>
+  <si>
+    <t>p_won20</t>
+  </si>
+  <si>
+    <t>p_wof1</t>
+  </si>
+  <si>
+    <t>p_wof2</t>
+  </si>
+  <si>
+    <t>p_wof3</t>
+  </si>
+  <si>
+    <t>p_wof4</t>
+  </si>
+  <si>
+    <t>p_wof5</t>
+  </si>
+  <si>
+    <t>p_wof6</t>
+  </si>
+  <si>
+    <t>p_wof7</t>
+  </si>
+  <si>
+    <t>p_wof8</t>
+  </si>
+  <si>
+    <t>p_wof9</t>
+  </si>
+  <si>
+    <t>p_wof10</t>
   </si>
   <si>
     <t>rez_spv_001</t>
@@ -1966,94 +1966,94 @@
     <t>e_sol20</t>
   </si>
   <si>
-    <t>e_won21</t>
-  </si>
-  <si>
-    <t>e_won22</t>
-  </si>
-  <si>
-    <t>e_won23</t>
-  </si>
-  <si>
-    <t>e_won24</t>
-  </si>
-  <si>
-    <t>e_won25</t>
-  </si>
-  <si>
-    <t>e_won26</t>
-  </si>
-  <si>
-    <t>e_won27</t>
-  </si>
-  <si>
-    <t>e_won28</t>
-  </si>
-  <si>
-    <t>e_won29</t>
-  </si>
-  <si>
-    <t>e_won30</t>
-  </si>
-  <si>
-    <t>e_won31</t>
-  </si>
-  <si>
-    <t>e_won32</t>
-  </si>
-  <si>
-    <t>e_won33</t>
-  </si>
-  <si>
-    <t>e_won34</t>
-  </si>
-  <si>
-    <t>e_won35</t>
-  </si>
-  <si>
-    <t>e_won36</t>
-  </si>
-  <si>
-    <t>e_won37</t>
-  </si>
-  <si>
-    <t>e_won38</t>
-  </si>
-  <si>
-    <t>e_won39</t>
-  </si>
-  <si>
-    <t>e_won40</t>
-  </si>
-  <si>
-    <t>e_wof41</t>
-  </si>
-  <si>
-    <t>e_wof42</t>
-  </si>
-  <si>
-    <t>e_wof43</t>
-  </si>
-  <si>
-    <t>e_wof44</t>
-  </si>
-  <si>
-    <t>e_wof45</t>
-  </si>
-  <si>
-    <t>e_wof46</t>
-  </si>
-  <si>
-    <t>e_wof47</t>
-  </si>
-  <si>
-    <t>e_wof48</t>
-  </si>
-  <si>
-    <t>e_wof49</t>
-  </si>
-  <si>
-    <t>e_wof50</t>
+    <t>e_won1</t>
+  </si>
+  <si>
+    <t>e_won2</t>
+  </si>
+  <si>
+    <t>e_won3</t>
+  </si>
+  <si>
+    <t>e_won4</t>
+  </si>
+  <si>
+    <t>e_won5</t>
+  </si>
+  <si>
+    <t>e_won6</t>
+  </si>
+  <si>
+    <t>e_won7</t>
+  </si>
+  <si>
+    <t>e_won8</t>
+  </si>
+  <si>
+    <t>e_won9</t>
+  </si>
+  <si>
+    <t>e_won10</t>
+  </si>
+  <si>
+    <t>e_won11</t>
+  </si>
+  <si>
+    <t>e_won12</t>
+  </si>
+  <si>
+    <t>e_won13</t>
+  </si>
+  <si>
+    <t>e_won14</t>
+  </si>
+  <si>
+    <t>e_won15</t>
+  </si>
+  <si>
+    <t>e_won16</t>
+  </si>
+  <si>
+    <t>e_won17</t>
+  </si>
+  <si>
+    <t>e_won18</t>
+  </si>
+  <si>
+    <t>e_won19</t>
+  </si>
+  <si>
+    <t>e_won20</t>
+  </si>
+  <si>
+    <t>e_wof1</t>
+  </si>
+  <si>
+    <t>e_wof2</t>
+  </si>
+  <si>
+    <t>e_wof3</t>
+  </si>
+  <si>
+    <t>e_wof4</t>
+  </si>
+  <si>
+    <t>e_wof5</t>
+  </si>
+  <si>
+    <t>e_wof6</t>
+  </si>
+  <si>
+    <t>e_wof7</t>
+  </si>
+  <si>
+    <t>e_wof8</t>
+  </si>
+  <si>
+    <t>e_wof9</t>
+  </si>
+  <si>
+    <t>e_wof10</t>
   </si>
   <si>
     <t>elc_spv_001</t>
@@ -2305,94 +2305,94 @@
     <t>POL-e_sol20</t>
   </si>
   <si>
-    <t>POL-e_won21</t>
-  </si>
-  <si>
-    <t>POL-e_won22</t>
-  </si>
-  <si>
-    <t>POL-e_won23</t>
-  </si>
-  <si>
-    <t>POL-e_won24</t>
-  </si>
-  <si>
-    <t>POL-e_won25</t>
-  </si>
-  <si>
-    <t>POL-e_won26</t>
-  </si>
-  <si>
-    <t>POL-e_won27</t>
-  </si>
-  <si>
-    <t>POL-e_won28</t>
-  </si>
-  <si>
-    <t>POL-e_won29</t>
-  </si>
-  <si>
-    <t>POL-e_won30</t>
-  </si>
-  <si>
-    <t>POL-e_won31</t>
-  </si>
-  <si>
-    <t>POL-e_won32</t>
-  </si>
-  <si>
-    <t>POL-e_won33</t>
-  </si>
-  <si>
-    <t>POL-e_won34</t>
-  </si>
-  <si>
-    <t>POL-e_won35</t>
-  </si>
-  <si>
-    <t>POL-e_won36</t>
-  </si>
-  <si>
-    <t>POL-e_won37</t>
-  </si>
-  <si>
-    <t>POL-e_won38</t>
-  </si>
-  <si>
-    <t>POL-e_won39</t>
-  </si>
-  <si>
-    <t>POL-e_won40</t>
-  </si>
-  <si>
-    <t>POL-e_wof41</t>
-  </si>
-  <si>
-    <t>POL-e_wof42</t>
-  </si>
-  <si>
-    <t>POL-e_wof43</t>
-  </si>
-  <si>
-    <t>POL-e_wof44</t>
-  </si>
-  <si>
-    <t>POL-e_wof45</t>
-  </si>
-  <si>
-    <t>POL-e_wof46</t>
-  </si>
-  <si>
-    <t>POL-e_wof47</t>
-  </si>
-  <si>
-    <t>POL-e_wof48</t>
-  </si>
-  <si>
-    <t>POL-e_wof49</t>
-  </si>
-  <si>
-    <t>POL-e_wof50</t>
+    <t>POL-e_won1</t>
+  </si>
+  <si>
+    <t>POL-e_won2</t>
+  </si>
+  <si>
+    <t>POL-e_won3</t>
+  </si>
+  <si>
+    <t>POL-e_won4</t>
+  </si>
+  <si>
+    <t>POL-e_won5</t>
+  </si>
+  <si>
+    <t>POL-e_won6</t>
+  </si>
+  <si>
+    <t>POL-e_won7</t>
+  </si>
+  <si>
+    <t>POL-e_won8</t>
+  </si>
+  <si>
+    <t>POL-e_won9</t>
+  </si>
+  <si>
+    <t>POL-e_won10</t>
+  </si>
+  <si>
+    <t>POL-e_won11</t>
+  </si>
+  <si>
+    <t>POL-e_won12</t>
+  </si>
+  <si>
+    <t>POL-e_won13</t>
+  </si>
+  <si>
+    <t>POL-e_won14</t>
+  </si>
+  <si>
+    <t>POL-e_won15</t>
+  </si>
+  <si>
+    <t>POL-e_won16</t>
+  </si>
+  <si>
+    <t>POL-e_won17</t>
+  </si>
+  <si>
+    <t>POL-e_won18</t>
+  </si>
+  <si>
+    <t>POL-e_won19</t>
+  </si>
+  <si>
+    <t>POL-e_won20</t>
+  </si>
+  <si>
+    <t>POL-e_wof1</t>
+  </si>
+  <si>
+    <t>POL-e_wof2</t>
+  </si>
+  <si>
+    <t>POL-e_wof3</t>
+  </si>
+  <si>
+    <t>POL-e_wof4</t>
+  </si>
+  <si>
+    <t>POL-e_wof5</t>
+  </si>
+  <si>
+    <t>POL-e_wof6</t>
+  </si>
+  <si>
+    <t>POL-e_wof7</t>
+  </si>
+  <si>
+    <t>POL-e_wof8</t>
+  </si>
+  <si>
+    <t>POL-e_wof9</t>
+  </si>
+  <si>
+    <t>POL-e_wof10</t>
   </si>
   <si>
     <t>POL-elc_spv_001</t>
@@ -26565,7 +26565,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FB12D24-450E-4344-8F32-4EAA16F84CD3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{943FEDA3-03AA-4618-8126-71B62465B096}">
   <dimension ref="B9:H120"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -26702,19 +26702,19 @@
         <v>482</v>
       </c>
       <c r="C16">
-        <v>55.043811628624923</v>
+        <v>51.599773363502067</v>
       </c>
       <c r="D16">
-        <v>17.297222745509313</v>
+        <v>21.56977526259324</v>
       </c>
       <c r="F16" t="s">
         <v>715</v>
       </c>
       <c r="G16">
-        <v>55.043811628624923</v>
+        <v>51.599773363502067</v>
       </c>
       <c r="H16">
-        <v>17.297222745509313</v>
+        <v>21.56977526259324</v>
       </c>
     </row>
     <row r="17" spans="2:8">
@@ -26722,19 +26722,19 @@
         <v>483</v>
       </c>
       <c r="C17">
-        <v>50.578080993739441</v>
+        <v>52.699096241559033</v>
       </c>
       <c r="D17">
-        <v>18.828842697375592</v>
+        <v>18.774188897221844</v>
       </c>
       <c r="F17" t="s">
         <v>716</v>
       </c>
       <c r="G17">
-        <v>50.578080993739441</v>
+        <v>52.699096241559033</v>
       </c>
       <c r="H17">
-        <v>18.828842697375592</v>
+        <v>18.774188897221844</v>
       </c>
     </row>
     <row r="18" spans="2:8">
@@ -26742,19 +26742,19 @@
         <v>484</v>
       </c>
       <c r="C18">
-        <v>51.683112043521319</v>
+        <v>50.596999579059187</v>
       </c>
       <c r="D18">
-        <v>21.60786681990249</v>
+        <v>18.767766636391777</v>
       </c>
       <c r="F18" t="s">
         <v>717</v>
       </c>
       <c r="G18">
-        <v>51.683112043521319</v>
+        <v>50.596999579059187</v>
       </c>
       <c r="H18">
-        <v>21.60786681990249</v>
+        <v>18.767766636391777</v>
       </c>
     </row>
     <row r="19" spans="2:8">
@@ -26762,19 +26762,19 @@
         <v>485</v>
       </c>
       <c r="C19">
-        <v>53.127919853895136</v>
+        <v>53.132136477480138</v>
       </c>
       <c r="D19">
-        <v>15.323117021697277</v>
+        <v>15.320564106329304</v>
       </c>
       <c r="F19" t="s">
         <v>718</v>
       </c>
       <c r="G19">
-        <v>53.127919853895136</v>
+        <v>53.132136477480138</v>
       </c>
       <c r="H19">
-        <v>15.323117021697277</v>
+        <v>15.320564106329304</v>
       </c>
     </row>
     <row r="20" spans="2:8">
@@ -26782,19 +26782,19 @@
         <v>486</v>
       </c>
       <c r="C20">
-        <v>52.644301743197701</v>
+        <v>55.054870829132881</v>
       </c>
       <c r="D20">
-        <v>18.798187470059847</v>
+        <v>17.274960774489102</v>
       </c>
       <c r="F20" t="s">
         <v>719</v>
       </c>
       <c r="G20">
-        <v>52.644301743197701</v>
+        <v>55.054870829132881</v>
       </c>
       <c r="H20">
-        <v>18.798187470059847</v>
+        <v>17.274960774489102</v>
       </c>
     </row>
     <row r="21" spans="2:8">
@@ -28803,7 +28803,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D92FF3B0-0FD0-4E7A-9CE8-6F9200981C73}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DFEC68E-C31C-4EC9-89FD-8DB00E6B26DF}">
   <dimension ref="B9:L120"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -29009,7 +29009,7 @@
         <v>587</v>
       </c>
       <c r="H16" t="s">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="J16" t="s">
         <v>596</v>
@@ -29038,7 +29038,7 @@
         <v>587</v>
       </c>
       <c r="H17" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="J17" t="s">
         <v>596</v>
@@ -29067,7 +29067,7 @@
         <v>587</v>
       </c>
       <c r="H18" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="J18" t="s">
         <v>596</v>
@@ -29125,7 +29125,7 @@
         <v>587</v>
       </c>
       <c r="H20" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="J20" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Updated POL_grids_syn_5 model - 2025-11-20 17:50
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{479ECF1D-3BA6-4E5D-87C4-74D2FD9F76AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E17475DF-D704-4101-BE09-830D807DA43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26565,7 +26565,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{943FEDA3-03AA-4618-8126-71B62465B096}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57CEB712-45E9-458B-A2D3-A3C19F566787}">
   <dimension ref="B9:H120"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28803,7 +28803,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DFEC68E-C31C-4EC9-89FD-8DB00E6B26DF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5392EBF1-FA90-4F07-94F6-CFC792D20E3D}">
   <dimension ref="B9:L120"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>